<commit_message>
Studio 2: nötr zemin ailesi — kâğıt beyazı #F5F5F5
Eski stüdyodaki açık zemin Studio 2'de yoktu; en açık iki zemin de sıcak
ya da zeytin tonluydu. Afişten ölçülen renk tam #F5F5F5, mürekkep saf
siyah. Üçüncü bir aile olarak eklendi:

  kâğıt  #F5F5F5  (mürekkep #000000)
  açık   #BEBEBE
  orta   #717171
  koyu   #3C3C3C
  siyah  #1E1E1E

Ara tonlar diğer ailelerle aynı L* basamaklarında türetildi (77 · 47,6 ·
25,3 · 11,3) — "orta" artık hangi aile seçilirse seçilsin aynı koyulukta.

ZEMİN sütunu da tanıyor: "NÖTR KÂĞIT", "NÖTR ORTA" vb. Şablondaki açılır
listeye beş değer eklendi.

Doğrulama: tuval rgb(245,245,245) / rgb(0,0,0); JPG çıktısının zemini de
245,245,245.
</commit_message>
<xml_diff>
--- a/public/sablon/kulalilar-afis-sablonu.xlsx
+++ b/public/sablon/kulalilar-afis-sablonu.xlsx
@@ -916,7 +916,7 @@
       <formula1>"1,2,3,4"</formula1>
     </dataValidation>
     <dataValidation sqref="N2:N405" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Geçersiz değer" error="Bu sütunda yalnız listedeki değerler kullanılabilir." type="list">
-      <formula1>"SICAK KÂĞIT,SICAK AÇIK,SICAK ORTA,SICAK KOYU,SICAK SİYAH,ZEYTİN KÂĞIT,ZEYTİN AÇIK,ZEYTİN ORTA,ZEYTİN KOYU,ZEYTİN SİYAH"</formula1>
+      <formula1>"NÖTR KÂĞIT,NÖTR AÇIK,NÖTR ORTA,NÖTR KOYU,NÖTR SİYAH,SICAK KÂĞIT,SICAK AÇIK,SICAK ORTA,SICAK KOYU,SICAK SİYAH,ZEYTİN KÂĞIT,ZEYTİN AÇIK,ZEYTİN ORTA,ZEYTİN KOYU,ZEYTİN SİYAH"</formula1>
     </dataValidation>
     <dataValidation sqref="P2:P405" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PANCAR DEPO,SÖKE FABRİKA SEVK,BOZÖYÜK SEVK"</formula1>
@@ -932,7 +932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1472,68 +1472,103 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SICAK KÂĞIT</t>
+          <t>NÖTR KÂĞIT</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SICAK AÇIK</t>
+          <t>NÖTR AÇIK</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>SICAK ORTA</t>
+          <t>NÖTR ORTA</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>SICAK KOYU</t>
+          <t>NÖTR KOYU</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>SICAK SİYAH</t>
+          <t>NÖTR SİYAH</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ZEYTİN KÂĞIT</t>
+          <t>SICAK KÂĞIT</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ZEYTİN AÇIK</t>
+          <t>SICAK AÇIK</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ZEYTİN ORTA</t>
+          <t>SICAK ORTA</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ZEYTİN KOYU</t>
+          <t>SICAK KOYU</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
+        <is>
+          <t>SICAK SİYAH</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>ZEYTİN KÂĞIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>ZEYTİN AÇIK</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>ZEYTİN ORTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>ZEYTİN KOYU</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
         <is>
           <t>ZEYTİN SİYAH</t>
         </is>

</xml_diff>